<commit_message>
sih: Sujitha off git (Canva-only Media & Design); role + milestone refresh
- Sujitha: E4 video + E5 deck in Canva/CapCut + SOC-UI mockups; hands files to
  the team, never touches the repo. E1/D5 (repo public, Drive link) -> Harish;
  E2 (README) -> Kaviya; portal submission text drafted by Archana.
- Milestone owners updated to match; Sep 19 submit -> Harish.
- SIH_TEAM_PLAN.md section 6: structured plan for teaching Manjari to attack
  (nmap/hping3/replay, lab-only rules, two mentored sessions, REDTEAM_SCENARIOS.md
  deliverable feeding D3).
- Live tracker sheet 1228SXz-... updated via build_sih_tracker.py --update.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFfmz2cueszq3uRNQ9VqLh
</commit_message>
<xml_diff>
--- a/scripts/sih_tracker_data/SIH26153_Team_Tracker.xlsx
+++ b/scripts/sih_tracker_data/SIH26153_Team_Tracker.xlsx
@@ -1285,17 +1285,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>harishvidyarthcsecs</t>
+          <t>harishvidyarth</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>R2, R7, D4</t>
+          <t>R2, R7, D4, D5, E1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>dual-head LSTM + K-step rollout; leakage-safe splits + per-class recall + retrain to a passing release gate (D4); LogReg benchmark (R7); CI, branch protection, release tag; mentors Manjari on the attack side</t>
+          <t>dual-head LSTM + K-step rollout; leakage-safe splits + per-class recall + retrain to a passing release gate (D4); LogReg benchmark (R7); CI, branch protection, release tag; make repo public / Drive code link (E1, D5); submit on the portal; mentors Manjari on the attack side</t>
         </is>
       </c>
     </row>
@@ -1322,12 +1322,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R6, E2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>FastAPI + Next.js cockpit + Streamlit; docker compose one-command demo; PCAP/CSV upload; STIX-lite alert + SOC PDF wiring (R6); owns Milestones tab + daily-report enforcement</t>
+          <t>FastAPI backend + no-build SOC UI; docker compose one-command demo; PCAP/CSV upload; STIX-lite alert + SOC PDF wiring (R6); README + setup instructions (E2); owns Milestones tab + daily-report enforcement</t>
         </is>
       </c>
     </row>
@@ -1427,23 +1427,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Media &amp; Submission</t>
+          <t>Media &amp; Design (no git)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PPT, frontend UI/UX</t>
+          <t>Canva, PPT, UI/UX</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>E1, E2, E4, E5 build, D5</t>
+          <t>E4 assets, E5 deck</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>builds the 5-slide deck + 2-min demo video; cockpit UI/UX polish; README polish; SIH portal submission text; make repo public / prepare Drive code link (D5)</t>
+          <t>5-slide deck in Canva (from docs/SLIDES.md); 2-min demo video edit in Canva / CapCut (from docs/DEMO_VIDEO_SCRIPT.md); SOC-UI mockups in Canva/Figma for a dev to implement; diagram polish for the architecture doc. Hands final files to the team — does not touch the repo.</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Kaviya / Harish / Sujitha</t>
+          <t>Kaviya / Harish</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2-min demo video (E4); 5-slide deck (E5); docker compose one-command demo on a clean machine; Manjari attack-training run</t>
+          <t>2-min demo video (E4, Sujitha in Canva); 5-slide deck (E5, Sujitha in Canva); docker compose one-command demo on a clean machine; Manjari attack-training run</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1618,12 +1618,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Buffer + polish; judge Q&amp;A prep; portal submission text; repo public / Drive link (E1, D5); pitch dry-run</t>
+          <t>Buffer + polish; judge Q&amp;A prep; portal submission text (Archana drafts); repo public / Drive link (E1, D5, Harish); pitch dry-run (Manjari)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Manjari (pitch) / Sujitha / all</t>
+          <t>Harish / Archana / Manjari</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sujitha (Harish confirms)</t>
+          <t>Harish</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Repo private + ~67 uncommitted working-tree changes -&gt; reproducibility / hygiene risk for judges</t>
+          <t>Repo hygiene: uncommitted WIP + XDR/response slice unstaged -&gt; reproducibility risk for judges</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sujitha</t>
+          <t>Harish</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>

<commit_message>
sih(tracker): fix E1/E2/E3/E4/E5 owners + evidence for the NIDS repo
E1 -> Harish (github.com/harishvidyarth/NIDS, confirm public / Drive fallback).
E2 -> Kaviya (README fresh-machine setup section).
E3 -> Archana, re-baselined 30% (raw material in reports/PIPELINE/PROTOTYPE; doc unwritten).
E4/E5 -> Sujitha in Canva; NAF script/slides not migrated, so both re-baselined low.
Pushed to live sheet 1228SXz-... via --update.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFfmz2cueszq3uRNQ9VqLh
</commit_message>
<xml_diff>
--- a/scripts/sih_tracker_data/SIH26153_Team_Tracker.xlsx
+++ b/scripts/sih_tracker_data/SIH26153_Team_Tracker.xlsx
@@ -1064,24 +1064,24 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sujitha</t>
+          <t>Harish</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>repo private</t>
+          <t>github.com/harishvidyarth/NIDS</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>make public / Drive zip (D5)</t>
+          <t>confirm repo public; prep Drive zip fallback (D5)</t>
         </is>
       </c>
     </row>
@@ -1098,24 +1098,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sujitha</t>
+          <t>Kaviya</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>80</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>README.md; README-OPS.md; DEMO_RUNBOOK.md</t>
+          <t>README.md</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>polish pass</t>
+          <t>add a fresh-machine setup section (.venv-lstm312, run_backend.sh, :8765)</t>
         </is>
       </c>
     </row>
@@ -1138,18 +1138,18 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>docs/ARCHITECTURE_NOTE.md</t>
+          <t>reports/NIDS_System_Guide_and_Roadmap.pdf; PIPELINE.md; PROTOTYPE.md</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>trim to 2 pp; single state story (D6)</t>
+          <t>write the 2-page judge-facing doc; single state story (D6)</t>
         </is>
       </c>
     </row>
@@ -1172,18 +1172,18 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>docs/DEMO_VIDEO_SCRIPT.md</t>
+          <t>-- (script not yet migrated from NAF)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>recording unverified</t>
+          <t>Sujitha edits in Canva / CapCut; script + recording both to do</t>
         </is>
       </c>
     </row>
@@ -1206,18 +1206,18 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>docs/SLIDES.md</t>
+          <t>reports/ figures + NIDS_Product_Description.pdf</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>deck unverified</t>
+          <t>Sujitha builds in Canva from reports/ + the E3 arch doc</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sih(tracker): Overview repo=NIDS; E1 link->Harish; E4/E5 links Sujitha builds, Harish posts
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFfmz2cueszq3uRNQ9VqLh
</commit_message>
<xml_diff>
--- a/scripts/sih_tracker_data/SIH26153_Team_Tracker.xlsx
+++ b/scripts/sih_tracker_data/SIH26153_Team_Tracker.xlsx
@@ -526,7 +526,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>github.com/harishvidyarthcsecs/network-attack-forecasting (private)</t>
+          <t>github.com/harishvidyarth/NIDS</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TBD — Sujitha</t>
+          <t>TBD — Harish</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TBD — Sujitha</t>
+          <t>TBD — Sujitha builds file, Harish posts link</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TBD — Sujitha</t>
+          <t>TBD — Sujitha builds deck, Harish posts link</t>
         </is>
       </c>
     </row>

</xml_diff>